<commit_message>
Auto-detect import type from Workday file metadata
Imports now auto-detect current vs historical period from file metadata
(period name in title row). Period ID and name auto-populate from the
file. Dashboard shows smarter empty state acknowledging historical data
when no current employees exist.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/sample-historical-2023-Q3.xlsx
+++ b/samples/sample-historical-2023-Q3.xlsx
@@ -413,538 +413,260 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:S54"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Associate Awards:: Compensation Review: Bonus - CY23 Q3</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Associate</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Supervisory Organization</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Current Job Profile</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Photo</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Errors</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Associate ID</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Current Base Pay All Countries</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Current Base Pay All Countries (USD)</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Grade</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Annual Bonus Target Percent</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Last Bonus Allocation Percent</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Bonus Target - Local Currency</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Bonus Target - Local Currency (USD)</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Proposed Bonus Amount</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Proposed Bonus Amount (USD)</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Proposed Percent of Target Bonus</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Zero Bonus Allocated</t>
+          <t>My Current Organizations Budget and Spend</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Della Gate</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Director)</t>
+          <t>Total Spend Text Value</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+          <t>of</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Total Pool Text Value</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>% Pool Spent</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MGR100</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>210000</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L3" t="n">
-        <v>85</v>
-      </c>
-      <c r="M3" t="n">
-        <v>9450</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>96.09999999999999</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Performance Rating: 100%</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr"/>
+          <t>Data Viz Color [Singular]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rhoda Map</t>
+          <t>Bonus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Director)</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+          <t>of</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>266152.5</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MGR101</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>205000</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>85</v>
-      </c>
-      <c r="M4" t="n">
-        <v>9225</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Performance Rating: 92%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Mai Stone
-Mentees: Sam Box
-Strengths: Fail Fast, Fix Faster, Delete More Than You Add, Tests or It's a Hallucination
-Areas for Improvement: Automate Yourself Out of a Job, Treat Servers Like Cattle, Not Pets, Sleep is a Feature</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
+          <t>style1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kay P. Eye</t>
+          <t>Compensation Planning Header</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Director)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>MGR102</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>215000</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L5" t="n">
-        <v>95</v>
-      </c>
-      <c r="M5" t="n">
-        <v>9675</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>106</v>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Performance Rating: 109%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Strengths: Be a Rubber Duck, Ship It to Learn It, Treat Servers Like Cattle, Not Pets
-Areas for Improvement: Blame the Process, Not the Person, Sleep is a Feature</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
+          <t>Compensation Planning</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Agie Enda</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Supervisory Organization (Director)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>MGR103</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>208000</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L6" t="n">
-        <v>85</v>
-      </c>
-      <c r="M6" t="n">
-        <v>9360</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>90.2</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Performance Rating: 92%
-Justification: Dependable team member who delivers consistently.
-Mentor: Mai Stone
-Mentees: Kenny Canary, Lou Pe
-Strengths: Automate Yourself Out of a Job, YAGNI (You Ain't Gonna Need It), Fail Fast, Fix Faster
-Areas for Improvement: Be a Rubber Duck, Ship It to Learn It</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
+          <t>Process Preferences</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mai Stone</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Supervisory Organization (Director)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>MGR104</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>212000</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L7" t="n">
-        <v>105</v>
-      </c>
-      <c r="M7" t="n">
-        <v>9540</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>108.8</v>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Performance Rating: 105%</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+          <t>Organization Issues</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Paige Duty</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Supervisory Organization (Della Gate)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Staff Software Developer</t>
-        </is>
-      </c>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EMP1000</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>190000</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>IC4</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L8" t="n">
-        <v>95</v>
-      </c>
-      <c r="M8" t="n">
-        <v>7125</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>92.59999999999999</v>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Performance Rating: 94%
-Justification: Dependable team member who delivers consistently.
-Mentor: Rhoda Map
-Strengths: Tests or It's a Hallucination, Strong Opinions, Loosely Held, YAGNI (You Ain't Gonna Need It)
-Areas for Improvement: Be a Rubber Duck, Ship It to Learn It</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>Bonus</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Lee Latency</t>
+          <t>Associate</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Supervisory Organization</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+          <t>Current Job Profile</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>EMP1001</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>180000</v>
+          <t>Associate ID</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Current Base Pay All Countries</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Current Base Pay All Countries (USD)</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>IC4</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L9" t="n">
-        <v>105</v>
-      </c>
-      <c r="M9" t="n">
-        <v>6750</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>111.4</v>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Annual Bonus Target %</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Last Bonus Allocation %</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Bonus Target - Local Currency</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Bonus Target - Local Currency (USD)</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Proposed Bonus Amount</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Proposed Bonus Amount (USD)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Proposed % of Target Bonus</t>
+        </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Performance Rating: 109%
-Justification: Dependable team member who delivers consistently.
-Mentor: Mai Stone
-Mentees: Lou Pe
-Strengths: Ship It to Learn It, Tests or It's a Hallucination, Fail Fast, Fix Faster
-Areas for Improvement: Be a Rubber Duck, Leave the Campfire Cleaner, Strong Opinions, Loosely Held</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Zero Bonus Allocated</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mona Torr</t>
+          <t>Della Gate</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>EMP1002</t>
+          <t>MGR100</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>175000</v>
+        <v>210000</v>
+      </c>
+      <c r="H10" t="n">
+        <v>210000</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -953,27 +675,28 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L10" t="n">
-        <v>110</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>6562.5</v>
-      </c>
+        <v>12600</v>
+      </c>
+      <c r="N10" t="n">
+        <v>12600</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>114.1</v>
+        <v>84</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Performance Rating: 110%
-Justification: Strong performance with notable achievements in code quality and team collaboration.
-Strengths: Comments are Apologies, Tests or It's a Hallucination, Sleep is a Feature
-Areas for Improvement: Be a Rubber Duck, Blame the Process, Not the Person</t>
+          <t>Performance Rating: 84%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -981,28 +704,31 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Robin Rollback</t>
+          <t>Paige Duty</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Principal Engineer</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>EMP1003</t>
+          <t>EMP2001</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>125000</v>
+        <v>220000</v>
+      </c>
+      <c r="H11" t="n">
+        <v>220000</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1011,24 +737,28 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC5</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="n">
-        <v>115</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>3750</v>
-      </c>
+        <v>11000</v>
+      </c>
+      <c r="N11" t="n">
+        <v>11000</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>94.5</v>
+        <v>73</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Performance Rating: 98%</t>
+          <t>Performance Rating: 73%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -1036,28 +766,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kenny Canary</t>
+          <t>Lee Latency</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Staff Software Developer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>EMP1004</t>
+          <t>EMP2002</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>145000</v>
+        <v>185000</v>
+      </c>
+      <c r="H12" t="n">
+        <v>185000</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1066,28 +799,28 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" t="n">
-        <v>115</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>4350</v>
-      </c>
+        <v>6937.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>6937.5</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>110.7</v>
+        <v>105</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Performance Rating: 110%
-Justification: Solid technical growth and increasing impact on team success.
-Mentor: Terry Byte
-Strengths: Fail Fast, Fix Faster, Comments are Apologies, Delete More Than You Add
-Areas for Improvement: Ship It to Learn It, Treat Servers Like Cattle, Not Pets, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 105%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -1095,28 +828,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tracey Loggins</t>
+          <t>Mona Torr</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Staff SRE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>EMP1005</t>
+          <t>EMP2003</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>120000</v>
+        <v>180000</v>
+      </c>
+      <c r="H13" t="n">
+        <v>180000</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1125,25 +861,28 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>2.5</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>3000</v>
-      </c>
+        <v>6750</v>
+      </c>
+      <c r="N13" t="n">
+        <v>6750</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>120.3</v>
+        <v>101</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Performance Rating: 117%
-Justification: Solid technical growth and increasing impact on team success.
-Mentor: Lee Latency
-Strengths: Be a Rubber Duck, Comments are Apologies, Ship It to Learn It
-Areas for Improvement: Automate Yourself Out of a Job, Leave the Campfire Cleaner, Treat Servers Like Cattle, Not Pets</t>
+          <t>Performance Rating: 101%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
@@ -1151,28 +890,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sue Q. Ell</t>
+          <t>Robin Rollback</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>EMP1006</t>
+          <t>EMP2004</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>115000</v>
+        <v>155000</v>
+      </c>
+      <c r="H14" t="n">
+        <v>155000</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1181,29 +923,28 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L14" t="n">
-        <v>105</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>2875</v>
-      </c>
+        <v>4650</v>
+      </c>
+      <c r="N14" t="n">
+        <v>4650</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>95.8</v>
+        <v>98</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Performance Rating: 93%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Terry Byte
-Mentees: Ty Po
-Strengths: Be a Rubber Duck, Sleep is a Feature, Comments are Apologies
-Areas for Improvement: Ship It to Learn It, Delete More Than You Add, Blame the Process, Not the Person</t>
+          <t>Performance Rating: 98%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
@@ -1211,28 +952,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jason Blob</t>
+          <t>Kenny Canary</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>EMP1007</t>
+          <t>EMP2005</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>118000</v>
+        <v>150000</v>
+      </c>
+      <c r="H15" t="n">
+        <v>150000</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1241,26 +985,28 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2.5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>2950</v>
-      </c>
+        <v>4500</v>
+      </c>
+      <c r="N15" t="n">
+        <v>4500</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>91.59999999999999</v>
+        <v>87</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Performance Rating: 91%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Al Ert
-Mentees: Sam Box, Robin Rollback
-Strengths: Treat Servers Like Cattle, Not Pets, Fail Fast, Fix Faster, Strong Opinions, Loosely Held
-Areas for Improvement: Delete More Than You Add, Sleep is a Feature</t>
+          <t>Performance Rating: 87%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -1268,12 +1014,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Al Ert</t>
+          <t>Tracey Loggins</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1285,11 +1031,14 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>EMP1008</t>
+          <t>EMP2006</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>112000</v>
+        <v>125000</v>
+      </c>
+      <c r="H16" t="n">
+        <v>125000</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1304,23 +1053,22 @@
       <c r="K16" t="n">
         <v>2.5</v>
       </c>
-      <c r="L16" t="n">
-        <v>115</v>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>2800</v>
-      </c>
+        <v>3125</v>
+      </c>
+      <c r="N16" t="n">
+        <v>3125</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>108.4</v>
+        <v>83</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Performance Rating: 107%
-Justification: Met all expectations. Reliable contributor with consistent delivery.
-Mentor: Kay P. Eye
-Mentees: Tim Out, Sam Box
-Strengths: Be a Rubber Duck, Comments are Apologies, Blame the Process, Not the Person
-Areas for Improvement: Tests or It's a Hallucination, Sleep is a Feature, Automate Yourself Out of a Job</t>
+          <t>Performance Rating: 83%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -1328,28 +1076,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Addie Min</t>
+          <t>Sue Q. Ell</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Della Gate)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>EMP1009</t>
+          <t>EMP2007</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>152000</v>
+        <v>120000</v>
+      </c>
+      <c r="H17" t="n">
+        <v>120000</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1358,29 +1109,28 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
-      </c>
-      <c r="L17" t="n">
-        <v>95</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>4560</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
-        <v>96.3</v>
+        <v>139</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Met all expectations. Reliable contributor with consistent delivery.
-Mentor: Lee Latency
-Mentees: Tim Out, Kenny Canary
-Strengths: YAGNI (You Ain't Gonna Need It), Delete More Than You Add, Ship It to Learn It
-Areas for Improvement: Treat Servers Like Cattle, Not Pets, Sleep is a Feature</t>
+          <t>Performance Rating: 139%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -1388,28 +1138,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tim Out</t>
+          <t>Addie Min</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>EMP1010</t>
+          <t>EMP2008</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>175000</v>
+        <v>160000</v>
+      </c>
+      <c r="H18" t="n">
+        <v>160000</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1418,28 +1171,28 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L18" t="n">
-        <v>90</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>6562.5</v>
-      </c>
+        <v>4800</v>
+      </c>
+      <c r="N18" t="n">
+        <v>4800</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="n">
-        <v>106.8</v>
+        <v>81</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Performance Rating: 106%
-Justification: Dependable team member who delivers consistently.
-Mentees: Kenny Canary, Pat Ch
-Strengths: Sleep is a Feature, Tests or It's a Hallucination, Ship It to Learn It
-Areas for Improvement: Blame the Process, Not the Person, YAGNI (You Ain't Gonna Need It)</t>
+          <t>Performance Rating: 81%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -1447,28 +1200,31 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Barbie Que</t>
+          <t>Jason Blob</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>EMP1011</t>
+          <t>EMP2009</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>172000</v>
+        <v>115000</v>
+      </c>
+      <c r="H19" t="n">
+        <v>115000</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1477,29 +1233,28 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L19" t="n">
-        <v>105</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>6450</v>
-      </c>
+        <v>2875</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2875</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Al Ert
-Mentees: Sam Box, Lou Pe
-Strengths: Ship It to Learn It, Comments are Apologies, Fail Fast, Fix Faster
-Areas for Improvement: Automate Yourself Out of a Job, Sleep is a Feature</t>
+          <t>Performance Rating: 124%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -1507,28 +1262,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Terry Byte</t>
+          <t>Al Ert</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Platform Engineering (Della Gate)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Junior Software Developer</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EMP1012</t>
+          <t>EMP2010</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>155000</v>
+        <v>95000</v>
+      </c>
+      <c r="H20" t="n">
+        <v>95000</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1537,29 +1295,28 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
-      </c>
-      <c r="L20" t="n">
-        <v>95</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>4650</v>
-      </c>
+        <v>1900</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1900</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
       <c r="Q20" t="n">
-        <v>94.2</v>
+        <v>74</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Dependable team member who delivers consistently.
-Mentor: Lee Latency
-Mentees: Pat Ch, Lou Pe
-Strengths: Tests or It's a Hallucination, Comments are Apologies, Fail Fast, Fix Faster
-Areas for Improvement: Blame the Process, Not the Person, Treat Servers Like Cattle, Not Pets, Delete More Than You Add</t>
+          <t>Performance Rating: 74%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -1567,28 +1324,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nole Pointer</t>
+          <t>Rhoda Map</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>EMP1013</t>
+          <t>MGR101</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>149000</v>
+        <v>205000</v>
+      </c>
+      <c r="H21" t="n">
+        <v>205000</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1597,28 +1357,28 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" t="n">
-        <v>85</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>4470</v>
-      </c>
+        <v>12300</v>
+      </c>
+      <c r="N21" t="n">
+        <v>12300</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
-        <v>107.9</v>
+        <v>73</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Performance Rating: 108%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Paige Duty
-Strengths: Delete More Than You Add, Tests or It's a Hallucination, Fail Fast, Fix Faster
-Areas for Improvement: Treat Servers Like Cattle, Not Pets, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 73%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -1626,28 +1386,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marge Conflict</t>
+          <t>Tim Out</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Principal Engineer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>EMP1014</t>
+          <t>EMP2011</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>110000</v>
+        <v>225000</v>
+      </c>
+      <c r="H22" t="n">
+        <v>225000</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1656,25 +1419,28 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC5</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>2.5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>2750</v>
-      </c>
+        <v>11250</v>
+      </c>
+      <c r="N22" t="n">
+        <v>11250</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="n">
-        <v>104.2</v>
+        <v>81</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Performance Rating: 102%
-Justification: Dependable team member who delivers consistently.
-Mentees: Jason Blob, Ty Po
-Strengths: Blame the Process, Not the Person, Tests or It's a Hallucination, Delete More Than You Add
-Areas for Improvement: Strong Opinions, Loosely Held, Sleep is a Feature</t>
+          <t>Performance Rating: 81%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -1682,28 +1448,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bridget Branch</t>
+          <t>Barbie Que</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Staff Software Developer</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>EMP1015</t>
+          <t>EMP2012</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>125000</v>
+        <v>190000</v>
+      </c>
+      <c r="H23" t="n">
+        <v>190000</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1712,25 +1481,28 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L23" t="n">
-        <v>90</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>3125</v>
-      </c>
+        <v>7125</v>
+      </c>
+      <c r="N23" t="n">
+        <v>7125</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="n">
-        <v>94.3</v>
+        <v>97</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Solid performance. Completed assigned work on time with good quality.</t>
+          <t>Performance Rating: 97%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -1738,12 +1510,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cody Ryder</t>
+          <t>Terry Byte</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1755,11 +1527,14 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>EMP1016</t>
+          <t>EMP2013</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>147000</v>
+        <v>160000</v>
+      </c>
+      <c r="H24" t="n">
+        <v>160000</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1774,19 +1549,22 @@
       <c r="K24" t="n">
         <v>3</v>
       </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>4410</v>
-      </c>
+        <v>4800</v>
+      </c>
+      <c r="N24" t="n">
+        <v>4800</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="n">
-        <v>90.59999999999999</v>
+        <v>99</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentees: Jason Blob
-Strengths: YAGNI (You Ain't Gonna Need It), Be a Rubber Duck, Blame the Process, Not the Person
-Areas for Improvement: Comments are Apologies, Delete More Than You Add</t>
+          <t>Performance Rating: 99%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
@@ -1794,28 +1572,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cy Ferr</t>
+          <t>Cody Ryder</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>EMP1017</t>
+          <t>EMP2014</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>122000</v>
+        <v>158000</v>
+      </c>
+      <c r="H25" t="n">
+        <v>158000</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1824,28 +1605,28 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K25" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L25" t="n">
-        <v>110</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>3050</v>
-      </c>
+        <v>4740</v>
+      </c>
+      <c r="N25" t="n">
+        <v>4740</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="n">
-        <v>98.7</v>
+        <v>134</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Performance Rating: 103%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Agie Enda
-Strengths: Leave the Campfire Cleaner, Blame the Process, Not the Person, YAGNI (You Ain't Gonna Need It)
-Areas for Improvement: Delete More Than You Add, Treat Servers Like Cattle, Not Pets, Be a Rubber Duck</t>
+          <t>Performance Rating: 134%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
@@ -1853,28 +1634,31 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Phil Wall</t>
+          <t>Nole Pointer</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>EMP1018</t>
+          <t>EMP2015</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>119000</v>
+        <v>155000</v>
+      </c>
+      <c r="H26" t="n">
+        <v>155000</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1883,29 +1667,28 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L26" t="n">
-        <v>100</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>2975</v>
-      </c>
+        <v>4650</v>
+      </c>
+      <c r="N26" t="n">
+        <v>4650</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="n">
-        <v>92.7</v>
+        <v>73</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Dependable team member who delivers consistently.
-Mentor: Agie Enda
-Mentees: Pat Ch, Kenny Canary
-Strengths: Delete More Than You Add, Strong Opinions, Loosely Held, YAGNI (You Ain't Gonna Need It)
-Areas for Improvement: Leave the Campfire Cleaner, Comments are Apologies, Treat Servers Like Cattle, Not Pets</t>
+          <t>Performance Rating: 73%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
@@ -1913,12 +1696,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lana Wan</t>
+          <t>Bridget Branch</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Rhoda Map)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1930,11 +1713,14 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>EMP1019</t>
+          <t>EMP2016</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>116000</v>
+        <v>120000</v>
+      </c>
+      <c r="H27" t="n">
+        <v>120000</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1949,18 +1735,22 @@
       <c r="K27" t="n">
         <v>2.5</v>
       </c>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>2900</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="N27" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="n">
-        <v>93.5</v>
+        <v>95</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Performance Rating: 96%
-Justification: Met all expectations. Reliable contributor with consistent delivery.
-Strengths: Be a Rubber Duck, Leave the Campfire Cleaner, Automate Yourself Out of a Job
-Areas for Improvement: Delete More Than You Add, Sleep is a Feature, Blame the Process, Not the Person</t>
+          <t>Performance Rating: 95%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
@@ -1968,12 +1758,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Artie Ficial</t>
+          <t>Cy Ferr</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1985,11 +1775,14 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>EMP1020</t>
+          <t>EMP2017</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>195000</v>
+        <v>118000</v>
+      </c>
+      <c r="H28" t="n">
+        <v>118000</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2004,22 +1797,22 @@
       <c r="K28" t="n">
         <v>2.5</v>
       </c>
-      <c r="L28" t="n">
-        <v>105</v>
-      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>4875</v>
-      </c>
+        <v>2950</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2950</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="n">
-        <v>82.8</v>
+        <v>139</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Performance Rating: 85%
-Justification: Technical skills developing but requires more focus on quality.
-Mentor: Kay P. Eye
-Strengths: Sleep is a Feature, YAGNI (You Ain't Gonna Need It), Fail Fast, Fix Faster
-Areas for Improvement: Be a Rubber Duck, Automate Yourself Out of a Job, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 139%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -2027,28 +1820,31 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ruth Cause</t>
+          <t>Lana Wan</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>EMP1021</t>
+          <t>EMP2018</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>182000</v>
+        <v>122000</v>
+      </c>
+      <c r="H29" t="n">
+        <v>122000</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2057,29 +1853,28 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L29" t="n">
-        <v>115</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>6825</v>
-      </c>
+        <v>3050</v>
+      </c>
+      <c r="N29" t="n">
+        <v>3050</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
-        <v>107.2</v>
+        <v>123</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Performance Rating: 108%
-Justification: Dependable team member who delivers consistently.
-Mentor: Agie Enda
-Mentees: Sam Box
-Strengths: Tests or It's a Hallucination, Comments are Apologies, Strong Opinions, Loosely Held
-Areas for Improvement: Sleep is a Feature, Leave the Campfire Cleaner, Delete More Than You Add</t>
+          <t>Performance Rating: 123%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
@@ -2087,28 +1882,31 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Matt Rick</t>
+          <t>Phil Wall</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Staff Software Developer</t>
+          <t>Junior Software Developer</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>EMP1022</t>
+          <t>EMP2019</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>178000</v>
+        <v>92000</v>
+      </c>
+      <c r="H30" t="n">
+        <v>92000</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2117,25 +1915,28 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L30" t="n">
-        <v>85</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>6675</v>
-      </c>
+        <v>1840</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1840</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="n">
-        <v>87.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Performance Rating: 90%
-Justification: Solid performance. Completed assigned work on time with good quality.</t>
+          <t>Performance Rating: 98%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
@@ -2143,28 +1944,31 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cassie Cache</t>
+          <t>Marge Conflict</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Frontend Experience (Rhoda Map)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>EMP1023</t>
+          <t>EMP2020</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>158000</v>
+        <v>125000</v>
+      </c>
+      <c r="H31" t="n">
+        <v>125000</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2173,29 +1977,28 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
-      </c>
-      <c r="L31" t="n">
-        <v>110</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>4740</v>
-      </c>
+        <v>3125</v>
+      </c>
+      <c r="N31" t="n">
+        <v>3125</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="n">
-        <v>109.1</v>
+        <v>127</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Performance Rating: 105%
-Justification: Dependable team member who delivers consistently.
-Mentor: Agie Enda
-Mentees: Pat Ch
-Strengths: Fail Fast, Fix Faster, Automate Yourself Out of a Job, Sleep is a Feature
-Areas for Improvement: Blame the Process, Not the Person, Be a Rubber Duck</t>
+          <t>Performance Rating: 127%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
@@ -2203,28 +2006,31 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sue Do</t>
+          <t>Kay P. Eye</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Senior Software Developer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>EMP1024</t>
+          <t>MGR102</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>152000</v>
+        <v>208000</v>
+      </c>
+      <c r="H32" t="n">
+        <v>208000</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2233,28 +2039,28 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="K32" t="n">
-        <v>3</v>
-      </c>
-      <c r="L32" t="n">
+        <v>6</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>12480</v>
+      </c>
+      <c r="N32" t="n">
+        <v>12480</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="n">
         <v>105</v>
       </c>
-      <c r="M32" t="n">
-        <v>4560</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>91.2</v>
-      </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Performance Rating: 92%
-Justification: Dependable team member who delivers consistently.
-Mentees: Robin Rollback
-Strengths: Tests or It's a Hallucination, Ship It to Learn It, Be a Rubber Duck
-Areas for Improvement: Blame the Process, Not the Person, Sleep is a Feature, YAGNI (You Ain't Gonna Need It)</t>
+          <t>Performance Rating: 105%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
@@ -2262,28 +2068,31 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pat Ch</t>
+          <t>Artie Ficial</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Principal Engineer</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>EMP1025</t>
+          <t>EMP2021</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>128000</v>
+        <v>230000</v>
+      </c>
+      <c r="H33" t="n">
+        <v>230000</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2292,22 +2101,28 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC5</t>
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2.5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
-        <v>3200</v>
-      </c>
+        <v>11500</v>
+      </c>
+      <c r="N33" t="n">
+        <v>11500</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="n">
-        <v>124.5</v>
+        <v>70</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Performance Rating: 125%
-Justification: Strong performance with notable achievements in code quality and team collaboration.</t>
+          <t>Performance Rating: 70%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
@@ -2315,28 +2130,31 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Devin Null</t>
+          <t>Ruth Cause</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Staff Software Developer</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>EMP1026</t>
+          <t>EMP2022</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>122000</v>
+        <v>188000</v>
+      </c>
+      <c r="H34" t="n">
+        <v>188000</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2345,29 +2163,28 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L34" t="n">
-        <v>100</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="n">
-        <v>3050</v>
-      </c>
+        <v>7050</v>
+      </c>
+      <c r="N34" t="n">
+        <v>7050</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
       <c r="Q34" t="n">
-        <v>107.1</v>
+        <v>90</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Performance Rating: 108%
-Justification: Dependable team member who delivers consistently.
-Mentor: Mai Stone
-Mentees: Tim Out, Ty Po
-Strengths: Ship It to Learn It, Strong Opinions, Loosely Held, Leave the Campfire Cleaner
-Areas for Improvement: Fail Fast, Fix Faster, YAGNI (You Ain't Gonna Need It)</t>
+          <t>Performance Rating: 90%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
@@ -2375,28 +2192,31 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Justin Time</t>
+          <t>Matt Rick</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Staff Software Developer</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>EMP1027</t>
+          <t>EMP2023</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>118000</v>
+        <v>185000</v>
+      </c>
+      <c r="H35" t="n">
+        <v>185000</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2405,27 +2225,28 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L35" t="n">
-        <v>95</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
-        <v>2950</v>
-      </c>
+        <v>6937.5</v>
+      </c>
+      <c r="N35" t="n">
+        <v>6937.5</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
       <c r="Q35" t="n">
-        <v>92.09999999999999</v>
+        <v>124</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Performance Rating: 90%
-Justification: Dependable team member who delivers consistently.
-Strengths: Treat Servers Like Cattle, Not Pets, Blame the Process, Not the Person, Leave the Campfire Cleaner
-Areas for Improvement: Fail Fast, Fix Faster, Sleep is a Feature, Comments are Apologies</t>
+          <t>Performance Rating: 124%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
@@ -2433,12 +2254,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Annie O'Maly</t>
+          <t>Cassie Cache</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2450,11 +2271,14 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>EMP1028</t>
+          <t>EMP2024</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>155000</v>
+        <v>162000</v>
+      </c>
+      <c r="H36" t="n">
+        <v>162000</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2469,20 +2293,22 @@
       <c r="K36" t="n">
         <v>3</v>
       </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="n">
-        <v>4650</v>
-      </c>
+        <v>4860</v>
+      </c>
+      <c r="N36" t="n">
+        <v>4860</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
       <c r="Q36" t="n">
-        <v>94.90000000000001</v>
+        <v>113</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Performance Rating: 92%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Mai Stone
-Mentees: Sam Box
-Strengths: Treat Servers Like Cattle, Not Pets, Sleep is a Feature, Delete More Than You Add
-Areas for Improvement: Comments are Apologies, Tests or It's a Hallucination</t>
+          <t>Performance Rating: 113%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
@@ -2490,28 +2316,31 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sam Box</t>
+          <t>Annie O'Maly</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Kay P. Eye)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>EMP1029</t>
+          <t>EMP2025</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>125000</v>
+        <v>165000</v>
+      </c>
+      <c r="H37" t="n">
+        <v>165000</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2520,29 +2349,28 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L37" t="n">
-        <v>85</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="n">
-        <v>3125</v>
-      </c>
+        <v>4950</v>
+      </c>
+      <c r="N37" t="n">
+        <v>4950</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
       <c r="Q37" t="n">
-        <v>92.5</v>
+        <v>105</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Performance Rating: 93%
-Justification: Met all expectations. Reliable contributor with consistent delivery.
-Mentor: Della Gate
-Mentees: Sam Box
-Strengths: Comments are Apologies, Treat Servers Like Cattle, Not Pets, Ship It to Learn It
-Areas for Improvement: Leave the Campfire Cleaner, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 105%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
@@ -2550,65 +2378,61 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Val Idation</t>
+          <t>Sue Do</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Senior Software Developer</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>EMP1030</t>
+          <t>EMP2026</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>62000</v>
+        <v>158000</v>
       </c>
       <c r="H38" t="n">
-        <v>89911</v>
+        <v>158000</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L38" t="n">
-        <v>115</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
-        <v>1550</v>
+        <v>4740</v>
       </c>
       <c r="N38" t="n">
-        <v>2247.775</v>
-      </c>
+        <v>4740</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
       <c r="Q38" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Performance Rating: 84%
-Justification: Technical skills developing but requires more focus on quality.
-Mentor: Agie Enda
-Mentees: Robin Rollback
-Strengths: Tests or It's a Hallucination, Comments are Apologies, Leave the Campfire Cleaner
-Areas for Improvement: Treat Servers Like Cattle, Not Pets, Blame the Process, Not the Person, Ship It to Learn It</t>
+          <t>Performance Rating: 89%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
@@ -2616,35 +2440,35 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bill Ding</t>
+          <t>Pat Ch</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>EMP1031</t>
+          <t>EMP2027</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>78000</v>
+        <v>128000</v>
       </c>
       <c r="H39" t="n">
-        <v>98734</v>
+        <v>128000</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2655,26 +2479,22 @@
       <c r="K39" t="n">
         <v>2.5</v>
       </c>
-      <c r="L39" t="n">
-        <v>95</v>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
-        <v>1950</v>
+        <v>3200</v>
       </c>
       <c r="N39" t="n">
-        <v>2468.35</v>
-      </c>
+        <v>3200</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
       <c r="Q39" t="n">
-        <v>103.1</v>
+        <v>97</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Performance Rating: 101%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Agie Enda
-Mentees: Lou Pe, Pat Ch
-Strengths: Leave the Campfire Cleaner, Ship It to Learn It, Strong Opinions, Loosely Held
-Areas for Improvement: YAGNI (You Ain't Gonna Need It), Comments are Apologies</t>
+          <t>Performance Rating: 97%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
@@ -2682,28 +2502,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ty Po</t>
+          <t>Devin Null</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Staff SRE</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>EMP1032</t>
+          <t>EMP2028</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>185000</v>
+        <v>124000</v>
+      </c>
+      <c r="H40" t="n">
+        <v>124000</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2712,27 +2535,28 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K40" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L40" t="n">
-        <v>105</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
-        <v>6937.5</v>
-      </c>
+        <v>3100</v>
+      </c>
+      <c r="N40" t="n">
+        <v>3100</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
       <c r="Q40" t="n">
-        <v>108.7</v>
+        <v>113</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Performance Rating: 108%
-Justification: Dependable team member who delivers consistently.
-Strengths: Ship It to Learn It, Sleep is a Feature, YAGNI (You Ain't Gonna Need It)
-Areas for Improvement: Blame the Process, Not the Person, Automate Yourself Out of a Job, Tests or It's a Hallucination</t>
+          <t>Performance Rating: 113%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
@@ -2740,28 +2564,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mike Roservices</t>
+          <t>Justin Time</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Staff SRE</t>
+          <t>Software Developer</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>EMP1033</t>
+          <t>EMP2029</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>183000</v>
+        <v>120000</v>
+      </c>
+      <c r="H41" t="n">
+        <v>120000</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2770,29 +2597,28 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L41" t="n">
-        <v>100</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="n">
-        <v>6862.5</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="N41" t="n">
+        <v>3000</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
       <c r="Q41" t="n">
-        <v>110.5</v>
+        <v>83</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Performance Rating: 109%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Paige Duty
-Mentees: Robin Rollback, Jason Blob
-Strengths: Ship It to Learn It, Comments are Apologies, Fail Fast, Fix Faster
-Areas for Improvement: Strong Opinions, Loosely Held, Be a Rubber Duck</t>
+          <t>Performance Rating: 83%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
@@ -2800,28 +2626,31 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Lou Pe</t>
+          <t>Sam Box</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Backend Services (Kay P. Eye)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Senior SRE</t>
+          <t>Junior Software Developer</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>EMP1034</t>
+          <t>EMP2030</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>155000</v>
+        <v>98000</v>
+      </c>
+      <c r="H42" t="n">
+        <v>98000</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2830,28 +2659,28 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
-      </c>
-      <c r="L42" t="n">
-        <v>95</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="n">
-        <v>4650</v>
-      </c>
+        <v>1960</v>
+      </c>
+      <c r="N42" t="n">
+        <v>1960</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
       <c r="Q42" t="n">
-        <v>94.3</v>
+        <v>81</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Performance Rating: 95%
-Justification: Dependable team member who delivers consistently.
-Mentees: Pat Ch, Sam Box
-Strengths: Sleep is a Feature, Be a Rubber Duck, YAGNI (You Ain't Gonna Need It)
-Areas for Improvement: Automate Yourself Out of a Job, Fail Fast, Fix Faster</t>
+          <t>Performance Rating: 81%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
@@ -2859,28 +2688,31 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Connie Tainer</t>
+          <t>Agie Enda</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Senior SRE</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>EMP1035</t>
+          <t>MGR103</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>152000</v>
+        <v>212000</v>
+      </c>
+      <c r="H43" t="n">
+        <v>212000</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2889,28 +2721,28 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
-      </c>
-      <c r="L43" t="n">
-        <v>115</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
-        <v>4560</v>
-      </c>
+        <v>12720</v>
+      </c>
+      <c r="N43" t="n">
+        <v>12720</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
       <c r="Q43" t="n">
-        <v>101.8</v>
+        <v>118</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Performance Rating: 98%
-Justification: Dependable team member who delivers consistently.
-Mentees: Sam Box, Tim Out
-Strengths: Treat Servers Like Cattle, Not Pets, Delete More Than You Add, Strong Opinions, Loosely Held
-Areas for Improvement: Leave the Campfire Cleaner, Fail Fast, Fix Faster, Ship It to Learn It</t>
+          <t>Performance Rating: 118%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
@@ -2918,28 +2750,31 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Noah Node</t>
+          <t>Ty Po</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Principal Engineer</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>EMP1036</t>
+          <t>EMP2031</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>125000</v>
+        <v>235000</v>
+      </c>
+      <c r="H44" t="n">
+        <v>235000</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2948,43 +2783,60 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC5</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>2.5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
-        <v>3125</v>
-      </c>
-      <c r="R44" t="inlineStr"/>
+        <v>11750</v>
+      </c>
+      <c r="N44" t="n">
+        <v>11750</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="n">
+        <v>82</v>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Performance Rating: 82%
+Justification: Sample historical data</t>
+        </is>
+      </c>
       <c r="S44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sara Ver</t>
+          <t>Mike Roservices</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Staff SRE</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>EMP1037</t>
+          <t>EMP2032</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>122000</v>
+        <v>192000</v>
+      </c>
+      <c r="H45" t="n">
+        <v>192000</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2993,26 +2845,28 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K45" t="n">
-        <v>2.5</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="n">
-        <v>3050</v>
-      </c>
+        <v>7200</v>
+      </c>
+      <c r="N45" t="n">
+        <v>7200</v>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
       <c r="Q45" t="n">
-        <v>104.4</v>
+        <v>115</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Performance Rating: 104%
-Justification: Dependable team member who delivers consistently.
-Mentor: Terry Byte
-Mentees: Jason Blob
-Strengths: YAGNI (You Ain't Gonna Need It), Comments are Apologies, Treat Servers Like Cattle, Not Pets
-Areas for Improvement: Be a Rubber Duck, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 115%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -3020,28 +2874,31 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Exa M. Elle</t>
+          <t>Val Idation</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Senior SRE</t>
+          <t>Staff SRE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>EMP1038</t>
+          <t>EMP2033</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>148000</v>
+        <v>195000</v>
+      </c>
+      <c r="H46" t="n">
+        <v>195000</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3050,29 +2907,28 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC4</t>
         </is>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
-      </c>
-      <c r="L46" t="n">
-        <v>105</v>
-      </c>
+        <v>3.75</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
       <c r="M46" t="n">
-        <v>4440</v>
-      </c>
+        <v>7312.5</v>
+      </c>
+      <c r="N46" t="n">
+        <v>7312.5</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
       <c r="Q46" t="n">
-        <v>93.90000000000001</v>
+        <v>114</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Performance Rating: 98%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Kay P. Eye
-Mentees: Tim Out, Kenny Canary
-Strengths: Treat Servers Like Cattle, Not Pets, Tests or It's a Hallucination, Strong Opinions, Loosely Held
-Areas for Improvement: Be a Rubber Duck, Ship It to Learn It</t>
+          <t>Performance Rating: 114%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
@@ -3080,28 +2936,31 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dee Ploi</t>
+          <t>Lou Pe</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Agie Enda)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Senior SRE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>EMP1039</t>
+          <t>EMP2034</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>130000</v>
+        <v>168000</v>
+      </c>
+      <c r="H47" t="n">
+        <v>168000</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -3110,28 +2969,28 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K47" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L47" t="n">
-        <v>115</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="n">
-        <v>3250</v>
-      </c>
+        <v>5040</v>
+      </c>
+      <c r="N47" t="n">
+        <v>5040</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
       <c r="Q47" t="n">
-        <v>100.6</v>
+        <v>103</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Performance Rating: 104%
-Justification: Dependable team member who delivers consistently.
-Mentees: Jason Blob, Lou Pe
-Strengths: YAGNI (You Ain't Gonna Need It), Automate Yourself Out of a Job, Sleep is a Feature
-Areas for Improvement: Leave the Campfire Cleaner, Delete More Than You Add</t>
+          <t>Performance Rating: 103%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
@@ -3139,28 +2998,31 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ray D. O'Button</t>
+          <t>Connie Tainer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Staff SRE</t>
+          <t>Senior SRE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>EMP1040</t>
+          <t>EMP2035</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>188000</v>
+        <v>162000</v>
+      </c>
+      <c r="H48" t="n">
+        <v>162000</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -3169,28 +3031,28 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L48" t="n">
-        <v>110</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
-        <v>7050</v>
-      </c>
+        <v>4860</v>
+      </c>
+      <c r="N48" t="n">
+        <v>4860</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
       <c r="Q48" t="n">
-        <v>98.3</v>
+        <v>75</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Performance Rating: 94%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentees: Jason Blob, Pat Ch
-Strengths: YAGNI (You Ain't Gonna Need It), Treat Servers Like Cattle, Not Pets, Strong Opinions, Loosely Held
-Areas for Improvement: Blame the Process, Not the Person, Sleep is a Feature</t>
+          <t>Performance Rating: 75%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S48" t="inlineStr"/>
@@ -3198,28 +3060,31 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Cam Elcase</t>
+          <t>Exa M. Elle</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Staff SRE</t>
+          <t>Senior SRE</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>EMP1041</t>
+          <t>EMP2036</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>186000</v>
+        <v>170000</v>
+      </c>
+      <c r="H49" t="n">
+        <v>170000</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3228,29 +3093,28 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>IC4</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="L49" t="n">
-        <v>115</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="n">
-        <v>6975</v>
-      </c>
+        <v>5100</v>
+      </c>
+      <c r="N49" t="n">
+        <v>5100</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
       <c r="Q49" t="n">
-        <v>114.1</v>
+        <v>128</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Performance Rating: 110%
-Justification: Exceeded expectations on key deliverables. Good balance of individual contribution and team support.
-Mentor: Al Ert
-Mentees: Robin Rollback, Jason Blob
-Strengths: Tests or It's a Hallucination, Delete More Than You Add, Comments are Apologies
-Areas for Improvement: Fail Fast, Fix Faster, Leave the Campfire Cleaner, Ship It to Learn It</t>
+          <t>Performance Rating: 128%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S49" t="inlineStr"/>
@@ -3258,28 +3122,31 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ben Chmark</t>
+          <t>Noah Node</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Senior SRE</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>EMP1043</t>
+          <t>EMP2037</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>156000</v>
+        <v>130000</v>
+      </c>
+      <c r="H50" t="n">
+        <v>130000</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3288,29 +3155,28 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>3</v>
-      </c>
-      <c r="L50" t="n">
-        <v>90</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="n">
-        <v>4680</v>
-      </c>
+        <v>3250</v>
+      </c>
+      <c r="N50" t="n">
+        <v>3250</v>
+      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
       <c r="Q50" t="n">
-        <v>111.8</v>
+        <v>138</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Performance Rating: 110%
-Justification: Solid technical growth and increasing impact on team success.
-Mentor: Della Gate
-Mentees: Sam Box
-Strengths: Fail Fast, Fix Faster, Treat Servers Like Cattle, Not Pets, Blame the Process, Not the Person
-Areas for Improvement: Delete More Than You Add, Tests or It's a Hallucination, Leave the Campfire Cleaner</t>
+          <t>Performance Rating: 138%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S50" t="inlineStr"/>
@@ -3318,28 +3184,31 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Grace Full</t>
+          <t>Sara Ver</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Senior SRE</t>
+          <t>SRE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>EMP1044</t>
+          <t>EMP2038</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>153000</v>
+        <v>125000</v>
+      </c>
+      <c r="H51" t="n">
+        <v>125000</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -3348,29 +3217,28 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>IC3</t>
+          <t>IC2</t>
         </is>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
-      </c>
-      <c r="L51" t="n">
-        <v>115</v>
-      </c>
+        <v>2.5</v>
+      </c>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="n">
-        <v>4590</v>
-      </c>
+        <v>3125</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3125</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
       <c r="Q51" t="n">
-        <v>89.3</v>
+        <v>85</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Performance Rating: 91%
-Justification: Met all expectations. Reliable contributor with consistent delivery.
-Mentor: Mai Stone
-Mentees: Sam Box
-Strengths: YAGNI (You Ain't Gonna Need It), Sleep is a Feature, Tests or It's a Hallucination
-Areas for Improvement: Be a Rubber Duck, Strong Opinions, Loosely Held</t>
+          <t>Performance Rating: 85%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S51" t="inlineStr"/>
@@ -3378,28 +3246,31 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Shel Script</t>
+          <t>Bill Ding</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Senior SRE</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>EMP1045</t>
+          <t>EMP2039</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>128000</v>
+        <v>165000</v>
+      </c>
+      <c r="H52" t="n">
+        <v>165000</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -3408,29 +3279,28 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>IC3</t>
         </is>
       </c>
       <c r="K52" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L52" t="n">
-        <v>90</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
-        <v>3200</v>
-      </c>
+        <v>4950</v>
+      </c>
+      <c r="N52" t="n">
+        <v>4950</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
       <c r="Q52" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Performance Rating: 108%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Mai Stone
-Mentees: Kenny Canary
-Strengths: Leave the Campfire Cleaner, Delete More Than You Add, Ship It to Learn It
-Areas for Improvement: Treat Servers Like Cattle, Not Pets, Comments are Apologies</t>
+          <t>Performance Rating: 118%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S52" t="inlineStr"/>
@@ -3438,12 +3308,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sal T. Hash</t>
+          <t>Dee Ploi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Infrastructure (Agie Enda)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3455,11 +3325,14 @@
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>EMP1046</t>
+          <t>EMP2040</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>124000</v>
+        <v>128000</v>
+      </c>
+      <c r="H53" t="n">
+        <v>128000</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -3474,20 +3347,22 @@
       <c r="K53" t="n">
         <v>2.5</v>
       </c>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="n">
-        <v>3100</v>
-      </c>
+        <v>3200</v>
+      </c>
+      <c r="N53" t="n">
+        <v>3200</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
       <c r="Q53" t="n">
-        <v>110.2</v>
+        <v>80</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Performance Rating: 106%
-Justification: Dependable team member who delivers consistently.
-Mentor: Terry Byte
-Mentees: Tim Out
-Strengths: Strong Opinions, Loosely Held, Sleep is a Feature, Fail Fast, Fix Faster
-Areas for Improvement: Tests or It's a Hallucination, Blame the Process, Not the Person</t>
+          <t>Performance Rating: 80%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S53" t="inlineStr"/>
@@ -3495,28 +3370,31 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Reba Boot</t>
+          <t>Mai Stone</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Supervisory Organization (Mai Stone)</t>
+          <t>Site Reliability (Mai Stone)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SRE</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>EMP1047</t>
+          <t>MGR104</t>
         </is>
       </c>
       <c r="G54" t="n">
-        <v>120000</v>
+        <v>215000</v>
+      </c>
+      <c r="H54" t="n">
+        <v>215000</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -3525,29 +3403,28 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>IC2</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="K54" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L54" t="n">
-        <v>100</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="n">
-        <v>3000</v>
-      </c>
+        <v>12900</v>
+      </c>
+      <c r="N54" t="n">
+        <v>12900</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
       <c r="Q54" t="n">
-        <v>104.5</v>
+        <v>140</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Performance Rating: 109%
-Justification: Solid performance. Completed assigned work on time with good quality.
-Mentor: Al Ert
-Mentees: Tim Out
-Strengths: Tests or It's a Hallucination, Delete More Than You Add, Automate Yourself Out of a Job
-Areas for Improvement: Comments are Apologies, YAGNI (You Ain't Gonna Need It)</t>
+          <t>Performance Rating: 140%
+Justification: Sample historical data</t>
         </is>
       </c>
       <c r="S54" t="inlineStr"/>

</xml_diff>